<commit_message>
add 'definition' columns to Excel template guide and config README
</commit_message>
<xml_diff>
--- a/examples/configuration_templates/pfa_config_template.xlsx
+++ b/examples/configuration_templates/pfa_config_template.xlsx
@@ -8,15 +8,15 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\smello\code\geoPFA\examples\configuration_templates\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C23B93D6-411E-4A34-9809-2442A82547E1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D022602E-2A10-4061-A185-A0502400B767}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="29520" yWindow="-10380" windowWidth="13830" windowHeight="7110" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="1080" yWindow="1080" windowWidth="18288" windowHeight="11028" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Configuration" sheetId="1" r:id="rId1"/>
     <sheet name="Guide" sheetId="2" r:id="rId2"/>
   </sheets>
-  <calcPr calcId="162913" iterateDelta="1E-4"/>
+  <calcPr calcId="162913"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -26,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="68" uniqueCount="43">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="85" uniqueCount="61">
   <si>
     <t>criteria</t>
   </si>
@@ -91,70 +91,124 @@
     <t>Required</t>
   </si>
   <si>
-    <t>Hierarchy name; blank continuation cells are forward-filled.</t>
-  </si>
-  <si>
     <t>Required numeric</t>
   </si>
   <si>
-    <t>Voter-veto criterion weight.</t>
-  </si>
-  <si>
-    <t>Voter-veto component weight.</t>
-  </si>
-  <si>
-    <t>Component prior probability.</t>
-  </si>
-  <si>
-    <t>Layer name and expected input filename stem.</t>
-  </si>
-  <si>
-    <t>Voter-veto layer weight.</t>
-  </si>
-  <si>
     <t>Required for combination</t>
   </si>
   <si>
-    <t>none, inverse, negate, ln, hill, or valley.</t>
-  </si>
-  <si>
     <t>Recommended</t>
   </si>
   <si>
-    <t>Workflow dispatch/documentation label.</t>
-  </si>
-  <si>
-    <t>Labels processed output.</t>
-  </si>
-  <si>
     <t>Conditional</t>
   </si>
   <si>
-    <t>Required by value-based processing; blank/none for geometry-only layers.</t>
-  </si>
-  <si>
-    <t>Required for CSV/TEC; embedded in shapefiles.</t>
-  </si>
-  <si>
     <t>x_col and y_col</t>
   </si>
   <si>
     <t>Conditional pair</t>
   </si>
   <si>
-    <t>Required for coordinate CSV/TEC; omit for shapefile or WKT geometry.</t>
-  </si>
-  <si>
-    <t>Required for a separate 3D coordinate column.</t>
-  </si>
-  <si>
-    <t>Required when vertical-reference conversion is needed.</t>
-  </si>
-  <si>
     <t>Optional</t>
   </si>
   <si>
-    <t>Free-text documentation.</t>
+    <t>Definition</t>
+  </si>
+  <si>
+    <t>Name of top-level PFA criterion</t>
+  </si>
+  <si>
+    <t>Organizes related components and corresponds to the criterion directory in structured input data folder. Blank continuation cells are forward-filled.</t>
+  </si>
+  <si>
+    <t>Numeric weight assigned to the criterion.</t>
+  </si>
+  <si>
+    <t>Used when combining multiple criteria to determine their relative contributions.</t>
+  </si>
+  <si>
+    <t>The name of a resource component within a criterion, such as heat, permeability, or infrastructure.</t>
+  </si>
+  <si>
+    <t>Every layer belongs to a component. In structured input data, this value should match the component directory name. In Excel, blank continuation cells are forward-filled.</t>
+  </si>
+  <si>
+    <t>The numeric weight assigned to a component.</t>
+  </si>
+  <si>
+    <t>Used when combining multiple components in a criterion  to determine their relative contributions.</t>
+  </si>
+  <si>
+    <t>The estimated prior probability that a component exists anywhere in the study area before data-layer evidence is applied.</t>
+  </si>
+  <si>
+    <t>Used by layer combination to establish the component’s prior favorability.</t>
+  </si>
+  <si>
+    <t>The name of an individual data or evidence layer.</t>
+  </si>
+  <si>
+    <t>Identifies the layer in the PFA dictionary. For structured input data, it should match the input file’s name without its extension.</t>
+  </si>
+  <si>
+    <t>The numeric weight assigned to an individual layer.</t>
+  </si>
+  <si>
+    <t>Determines the layer’s relative contribution when layers are combined within a component.</t>
+  </si>
+  <si>
+    <t>The mathematical transformation applied to processed layer values before layer combination.</t>
+  </si>
+  <si>
+    <t>Use none when values should remain unchanged. Supported methods are none, inverse, negate, ln, hill, and valley. Case-insensitive forms of none and JSON null represent no transformation. See geopfa.transformation.transform for info.</t>
+  </si>
+  <si>
+    <t>A label describing the processing operation intended for the layer.</t>
+  </si>
+  <si>
+    <t>Optionally used by workflow code for processing dispatch or documentation. The Excel-to-JSON converter stores this value but does not execute the processing operation.</t>
+  </si>
+  <si>
+    <t>The measurement units of the configured data values.</t>
+  </si>
+  <si>
+    <t>For documenting the input layer and is used by several processing functions when labeling output.</t>
+  </si>
+  <si>
+    <t>The name of the input attribute column containing values to process.</t>
+  </si>
+  <si>
+    <t>Required for value-based interpolation, kriging, polygon aggregation, and 3D-to-2D aggregation. It may be blank, omitted, or none for geometry-only operations such as unweighted distance or density calculations.</t>
+  </si>
+  <si>
+    <t>The coordinate reference system of the input coordinates, generally expressed as an EPSG code.</t>
+  </si>
+  <si>
+    <t>Required for CSV and TEC inputs that must be converted into spatial geometry. Shapefiles normally include CRS information internally, although documenting it may still be useful.</t>
+  </si>
+  <si>
+    <t>Name of the input columns containing X and Y or longitude and latitude coordinates.</t>
+  </si>
+  <si>
+    <t>Used for coordinate-based CSV or TEC input. Omit for shapefiles or WKT geometry input.</t>
+  </si>
+  <si>
+    <t>Name of the input column containing Z, elevation, or depth coordinates.</t>
+  </si>
+  <si>
+    <t>Required when 3D coordinates are stored in a separate column.</t>
+  </si>
+  <si>
+    <t>Vertical measurement unit or reference system associated with Z values.</t>
+  </si>
+  <si>
+    <t>Used when vertical-reference conversion is needed. Supported conversion references are m-msl, ft-msl, and epsg:&lt;integer&gt;.</t>
+  </si>
+  <si>
+    <t>Free-text information about the layer or its configuration.</t>
+  </si>
+  <si>
+    <t>Used for human-readable documentation; not interpreted by the converter.</t>
   </si>
 </sst>
 </file>
@@ -211,9 +265,15 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -562,200 +622,264 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{36350C53-10DF-40B8-A514-0EA653A43886}">
-  <dimension ref="A1:C17"/>
+  <dimension ref="A1:D19"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="13.77734375" customWidth="1"/>
-    <col min="2" max="2" width="13.88671875" customWidth="1"/>
-    <col min="3" max="3" width="67.5546875" customWidth="1"/>
+    <col min="1" max="1" width="18.77734375" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="37.77734375" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="13.33203125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="67.109375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A1" s="1" t="s">
+    <row r="1" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A1" s="2" t="s">
         <v>17</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="B1" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="C1" s="2" t="s">
         <v>18</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="D1" s="2" t="s">
         <v>19</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A2" t="s">
+    <row r="2" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A2" s="3" t="s">
         <v>0</v>
       </c>
-      <c r="B2" t="s">
+      <c r="B2" s="3" t="s">
+        <v>29</v>
+      </c>
+      <c r="C2" s="3" t="s">
         <v>20</v>
       </c>
-      <c r="C2" t="s">
+      <c r="D2" s="3" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A3" s="3" t="s">
+        <v>1</v>
+      </c>
+      <c r="B3" s="3" t="s">
+        <v>31</v>
+      </c>
+      <c r="C3" s="3" t="s">
         <v>21</v>
       </c>
-    </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A3" t="s">
-        <v>1</v>
-      </c>
-      <c r="B3" t="s">
+      <c r="D3" s="3" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4" ht="43.2" x14ac:dyDescent="0.3">
+      <c r="A4" s="3" t="s">
+        <v>2</v>
+      </c>
+      <c r="B4" s="3" t="s">
+        <v>33</v>
+      </c>
+      <c r="C4" s="3" t="s">
+        <v>20</v>
+      </c>
+      <c r="D4" s="3" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="5" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A5" s="3" t="s">
+        <v>3</v>
+      </c>
+      <c r="B5" s="3" t="s">
+        <v>35</v>
+      </c>
+      <c r="C5" s="3" t="s">
+        <v>21</v>
+      </c>
+      <c r="D5" s="3" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="6" spans="1:4" ht="43.2" x14ac:dyDescent="0.3">
+      <c r="A6" s="3" t="s">
+        <v>4</v>
+      </c>
+      <c r="B6" s="3" t="s">
+        <v>37</v>
+      </c>
+      <c r="C6" s="3" t="s">
+        <v>21</v>
+      </c>
+      <c r="D6" s="3" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="7" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A7" s="3" t="s">
+        <v>5</v>
+      </c>
+      <c r="B7" s="3" t="s">
+        <v>39</v>
+      </c>
+      <c r="C7" s="3" t="s">
+        <v>20</v>
+      </c>
+      <c r="D7" s="3" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="8" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A8" s="3" t="s">
+        <v>6</v>
+      </c>
+      <c r="B8" s="3" t="s">
+        <v>41</v>
+      </c>
+      <c r="C8" s="3" t="s">
+        <v>21</v>
+      </c>
+      <c r="D8" s="3" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="9" spans="1:4" ht="43.2" x14ac:dyDescent="0.3">
+      <c r="A9" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="B9" s="3" t="s">
+        <v>43</v>
+      </c>
+      <c r="C9" s="3" t="s">
         <v>22</v>
       </c>
-      <c r="C3" t="s">
+      <c r="D9" s="3" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="10" spans="1:4" ht="43.2" x14ac:dyDescent="0.3">
+      <c r="A10" s="3" t="s">
+        <v>15</v>
+      </c>
+      <c r="B10" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="C10" s="3" t="s">
         <v>23</v>
       </c>
-    </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A4" t="s">
-        <v>2</v>
-      </c>
-      <c r="B4" t="s">
-        <v>20</v>
-      </c>
-      <c r="C4" t="s">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A5" t="s">
-        <v>3</v>
-      </c>
-      <c r="B5" t="s">
-        <v>22</v>
-      </c>
-      <c r="C5" t="s">
+      <c r="D10" s="3" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="11" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A11" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="B11" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="C11" s="3" t="s">
+        <v>23</v>
+      </c>
+      <c r="D11" s="3" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="12" spans="1:4" ht="43.2" x14ac:dyDescent="0.3">
+      <c r="A12" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="B12" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="C12" s="3" t="s">
         <v>24</v>
       </c>
-    </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A6" t="s">
-        <v>4</v>
-      </c>
-      <c r="B6" t="s">
-        <v>22</v>
-      </c>
-      <c r="C6" t="s">
+      <c r="D12" s="3" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="13" spans="1:4" ht="43.2" x14ac:dyDescent="0.3">
+      <c r="A13" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="B13" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="C13" s="3" t="s">
+        <v>24</v>
+      </c>
+      <c r="D13" s="3" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="14" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A14" s="3" t="s">
         <v>25</v>
       </c>
-    </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A7" t="s">
-        <v>5</v>
-      </c>
-      <c r="B7" t="s">
-        <v>20</v>
-      </c>
-      <c r="C7" t="s">
+      <c r="B14" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="C14" s="3" t="s">
         <v>26</v>
       </c>
-    </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A8" t="s">
-        <v>6</v>
-      </c>
-      <c r="B8" t="s">
-        <v>22</v>
-      </c>
-      <c r="C8" t="s">
+      <c r="D14" s="3" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="15" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A15" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="B15" s="3" t="s">
+        <v>55</v>
+      </c>
+      <c r="C15" s="3" t="s">
+        <v>24</v>
+      </c>
+      <c r="D15" s="3" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="16" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A16" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="B16" s="3" t="s">
+        <v>57</v>
+      </c>
+      <c r="C16" s="3" t="s">
+        <v>24</v>
+      </c>
+      <c r="D16" s="3" t="s">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="17" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A17" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="B17" s="3" t="s">
+        <v>59</v>
+      </c>
+      <c r="C17" s="3" t="s">
         <v>27</v>
       </c>
-    </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A9" t="s">
-        <v>14</v>
-      </c>
-      <c r="B9" t="s">
-        <v>28</v>
-      </c>
-      <c r="C9" t="s">
-        <v>29</v>
-      </c>
-    </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A10" t="s">
-        <v>15</v>
-      </c>
-      <c r="B10" t="s">
-        <v>30</v>
-      </c>
-      <c r="C10" t="s">
-        <v>31</v>
-      </c>
-    </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A11" t="s">
-        <v>7</v>
-      </c>
-      <c r="B11" t="s">
-        <v>30</v>
-      </c>
-      <c r="C11" t="s">
-        <v>32</v>
-      </c>
-    </row>
-    <row r="12" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A12" t="s">
-        <v>8</v>
-      </c>
-      <c r="B12" t="s">
-        <v>33</v>
-      </c>
-      <c r="C12" t="s">
-        <v>34</v>
-      </c>
-    </row>
-    <row r="13" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A13" t="s">
-        <v>12</v>
-      </c>
-      <c r="B13" t="s">
-        <v>33</v>
-      </c>
-      <c r="C13" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="14" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A14" t="s">
-        <v>36</v>
-      </c>
-      <c r="B14" t="s">
-        <v>37</v>
-      </c>
-      <c r="C14" t="s">
-        <v>38</v>
-      </c>
-    </row>
-    <row r="15" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A15" t="s">
-        <v>11</v>
-      </c>
-      <c r="B15" t="s">
-        <v>33</v>
-      </c>
-      <c r="C15" t="s">
-        <v>39</v>
-      </c>
-    </row>
-    <row r="16" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A16" t="s">
-        <v>13</v>
-      </c>
-      <c r="B16" t="s">
-        <v>33</v>
-      </c>
-      <c r="C16" t="s">
-        <v>40</v>
-      </c>
-    </row>
-    <row r="17" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A17" t="s">
-        <v>16</v>
-      </c>
-      <c r="B17" t="s">
-        <v>41</v>
-      </c>
-      <c r="C17" t="s">
-        <v>42</v>
-      </c>
+      <c r="D17" s="3" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="18" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A18" s="3"/>
+      <c r="B18" s="3"/>
+      <c r="C18" s="3"/>
+      <c r="D18" s="3"/>
+    </row>
+    <row r="19" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A19" s="3"/>
+      <c r="B19" s="3"/>
+      <c r="C19" s="3"/>
+      <c r="D19" s="3"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
adjust units and transformation_method language in config README and template
</commit_message>
<xml_diff>
--- a/examples/configuration_templates/pfa_config_template.xlsx
+++ b/examples/configuration_templates/pfa_config_template.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\smello\code\geoPFA\examples\configuration_templates\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D022602E-2A10-4061-A185-A0502400B767}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{23BC7ED5-2697-4697-9F92-C5B232342934}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="1080" yWindow="1080" windowWidth="18288" windowHeight="11028" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="8520" yWindow="-15495" windowWidth="16245" windowHeight="11235" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Configuration" sheetId="1" r:id="rId1"/>
@@ -157,12 +157,6 @@
     <t>Determines the layer’s relative contribution when layers are combined within a component.</t>
   </si>
   <si>
-    <t>The mathematical transformation applied to processed layer values before layer combination.</t>
-  </si>
-  <si>
-    <t>Use none when values should remain unchanged. Supported methods are none, inverse, negate, ln, hill, and valley. Case-insensitive forms of none and JSON null represent no transformation. See geopfa.transformation.transform for info.</t>
-  </si>
-  <si>
     <t>A label describing the processing operation intended for the layer.</t>
   </si>
   <si>
@@ -172,9 +166,6 @@
     <t>The measurement units of the configured data values.</t>
   </si>
   <si>
-    <t>For documenting the input layer and is used by several processing functions when labeling output.</t>
-  </si>
-  <si>
     <t>The name of the input attribute column containing values to process.</t>
   </si>
   <si>
@@ -209,6 +200,15 @@
   </si>
   <si>
     <t>Used for human-readable documentation; not interpreted by the converter.</t>
+  </si>
+  <si>
+    <t>For documenting the input layer and is used for labeling the color bar or labels in outputs.</t>
+  </si>
+  <si>
+    <t>The mathematical transformation applied to map processed layer values to favorability before combination.</t>
+  </si>
+  <si>
+    <t>Use none when values should remain unchanged (e.g., wehn higher data values are direct indicators of higher favorability). Supported methods are none, inverse, negate, ln, hill, and valley. Case-insensitive forms of none and JSON null represent no transformation. See geopfa.transformation.transform for info.</t>
   </si>
 </sst>
 </file>
@@ -625,10 +625,10 @@
   <dimension ref="A1:D19"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="18.77734375" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="24.109375" customWidth="1"/>
     <col min="2" max="2" width="37.77734375" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="13.33203125" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="67.109375" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="14.44140625" customWidth="1"/>
+    <col min="4" max="4" width="72.44140625" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:4" x14ac:dyDescent="0.3">
@@ -743,18 +743,18 @@
         <v>42</v>
       </c>
     </row>
-    <row r="9" spans="1:4" ht="43.2" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:4" ht="58.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A9" s="3" t="s">
         <v>14</v>
       </c>
       <c r="B9" s="3" t="s">
-        <v>43</v>
+        <v>59</v>
       </c>
       <c r="C9" s="3" t="s">
         <v>22</v>
       </c>
       <c r="D9" s="3" t="s">
-        <v>44</v>
+        <v>60</v>
       </c>
     </row>
     <row r="10" spans="1:4" ht="43.2" x14ac:dyDescent="0.3">
@@ -762,13 +762,13 @@
         <v>15</v>
       </c>
       <c r="B10" s="3" t="s">
-        <v>45</v>
+        <v>43</v>
       </c>
       <c r="C10" s="3" t="s">
         <v>23</v>
       </c>
       <c r="D10" s="3" t="s">
-        <v>46</v>
+        <v>44</v>
       </c>
     </row>
     <row r="11" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
@@ -776,13 +776,13 @@
         <v>7</v>
       </c>
       <c r="B11" s="3" t="s">
-        <v>47</v>
+        <v>45</v>
       </c>
       <c r="C11" s="3" t="s">
         <v>23</v>
       </c>
       <c r="D11" s="3" t="s">
-        <v>48</v>
+        <v>58</v>
       </c>
     </row>
     <row r="12" spans="1:4" ht="43.2" x14ac:dyDescent="0.3">
@@ -790,13 +790,13 @@
         <v>8</v>
       </c>
       <c r="B12" s="3" t="s">
-        <v>49</v>
+        <v>46</v>
       </c>
       <c r="C12" s="3" t="s">
         <v>24</v>
       </c>
       <c r="D12" s="3" t="s">
-        <v>50</v>
+        <v>47</v>
       </c>
     </row>
     <row r="13" spans="1:4" ht="43.2" x14ac:dyDescent="0.3">
@@ -804,13 +804,13 @@
         <v>12</v>
       </c>
       <c r="B13" s="3" t="s">
-        <v>51</v>
+        <v>48</v>
       </c>
       <c r="C13" s="3" t="s">
         <v>24</v>
       </c>
       <c r="D13" s="3" t="s">
-        <v>52</v>
+        <v>49</v>
       </c>
     </row>
     <row r="14" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
@@ -818,13 +818,13 @@
         <v>25</v>
       </c>
       <c r="B14" s="3" t="s">
-        <v>53</v>
+        <v>50</v>
       </c>
       <c r="C14" s="3" t="s">
         <v>26</v>
       </c>
       <c r="D14" s="3" t="s">
-        <v>54</v>
+        <v>51</v>
       </c>
     </row>
     <row r="15" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
@@ -832,13 +832,13 @@
         <v>11</v>
       </c>
       <c r="B15" s="3" t="s">
-        <v>55</v>
+        <v>52</v>
       </c>
       <c r="C15" s="3" t="s">
         <v>24</v>
       </c>
       <c r="D15" s="3" t="s">
-        <v>56</v>
+        <v>53</v>
       </c>
     </row>
     <row r="16" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
@@ -846,13 +846,13 @@
         <v>13</v>
       </c>
       <c r="B16" s="3" t="s">
-        <v>57</v>
+        <v>54</v>
       </c>
       <c r="C16" s="3" t="s">
         <v>24</v>
       </c>
       <c r="D16" s="3" t="s">
-        <v>58</v>
+        <v>55</v>
       </c>
     </row>
     <row r="17" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
@@ -860,13 +860,13 @@
         <v>16</v>
       </c>
       <c r="B17" s="3" t="s">
-        <v>59</v>
+        <v>56</v>
       </c>
       <c r="C17" s="3" t="s">
         <v>27</v>
       </c>
       <c r="D17" s="3" t="s">
-        <v>60</v>
+        <v>57</v>
       </c>
     </row>
     <row r="18" spans="1:4" x14ac:dyDescent="0.3">

</xml_diff>